<commit_message>
data(W28): refresh other_channels sales for AA + Nexlev
Operator re-exported sales tab in both W28 other_channels.xlsx files.
Structure unchanged; sales sheet only.  Downstream sales_auto_etl will
re-emit W28 sales rows on next Weekly Auto-Sync.
</commit_message>
<xml_diff>
--- a/data/raw/sales/Week 28/Audio_Array/other_channels.xlsx
+++ b/data/raw/sales/Week 28/Audio_Array/other_channels.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Hazique Backup\Week 17\Week 28\raw\sales\Week 28\Audio_Array\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\raw\sales\Week 28\Audio_Array\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52916F30-A673-472F-B72E-BFD6021A9CF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E86B6F3-D604-46E9-BFB8-D737B208C4B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="D2C - Audio Array" sheetId="4" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="243">
   <si>
     <t>SKU</t>
   </si>
@@ -304,18 +304,12 @@
     <t>FBA76862</t>
   </si>
   <si>
-    <t>B0BPLWW72Y</t>
-  </si>
-  <si>
     <t>AM-C28</t>
   </si>
   <si>
     <t>TBLB</t>
   </si>
   <si>
-    <t>Enertia</t>
-  </si>
-  <si>
     <t>FBA79813</t>
   </si>
   <si>
@@ -334,18 +328,6 @@
     <t>AM-C2</t>
   </si>
   <si>
-    <t>AAFT ELEARN Private Limited</t>
-  </si>
-  <si>
-    <t>FBA79957</t>
-  </si>
-  <si>
-    <t>B0G3Q517Y2</t>
-  </si>
-  <si>
-    <t>AM-W23</t>
-  </si>
-  <si>
     <t>FBA80085</t>
   </si>
   <si>
@@ -355,30 +337,15 @@
     <t>M6</t>
   </si>
   <si>
-    <t>COMPUTER GALLERY</t>
-  </si>
-  <si>
     <t>FBA79009</t>
   </si>
   <si>
-    <t>B0CH4PMR8K</t>
-  </si>
-  <si>
     <t>AM-C41</t>
   </si>
   <si>
-    <t>EIS TECHINFRA SOLUTIONS INDIA P</t>
-  </si>
-  <si>
-    <t>Option</t>
-  </si>
-  <si>
     <t>FBA75692</t>
   </si>
   <si>
-    <t>B0B4G1HPL5</t>
-  </si>
-  <si>
     <t>AM-C11</t>
   </si>
   <si>
@@ -388,18 +355,9 @@
     <t>FBA78960</t>
   </si>
   <si>
-    <t>B0CBCB82MT</t>
-  </si>
-  <si>
     <t>AM-C39</t>
   </si>
   <si>
-    <t>FBA79816</t>
-  </si>
-  <si>
-    <t>B0FPR962YS</t>
-  </si>
-  <si>
     <t>FBA79999</t>
   </si>
   <si>
@@ -409,36 +367,6 @@
     <t>JTG800</t>
   </si>
   <si>
-    <t>FBA80000</t>
-  </si>
-  <si>
-    <t>B0GW8XGPB2</t>
-  </si>
-  <si>
-    <t>DP-718H</t>
-  </si>
-  <si>
-    <t>FBA80001</t>
-  </si>
-  <si>
-    <t>B0GW92TQGV</t>
-  </si>
-  <si>
-    <t>USB718</t>
-  </si>
-  <si>
-    <t>FBA80004</t>
-  </si>
-  <si>
-    <t>B0GW92316G</t>
-  </si>
-  <si>
-    <t>AM-W36 Pro</t>
-  </si>
-  <si>
-    <t>DIGIWAVES SOLUTIONS</t>
-  </si>
-  <si>
     <t>FBA79482</t>
   </si>
   <si>
@@ -671,13 +599,181 @@
   </si>
   <si>
     <t>AM-C40</t>
+  </si>
+  <si>
+    <t>B0B4G8ZB64</t>
+  </si>
+  <si>
+    <t>Enertia Worldwide Private Limit</t>
+  </si>
+  <si>
+    <t>Basil Industries</t>
+  </si>
+  <si>
+    <t>B0B4G763WS</t>
+  </si>
+  <si>
+    <t>B0B4G59Y8W</t>
+  </si>
+  <si>
+    <t>B0CH4T2BJD</t>
+  </si>
+  <si>
+    <t>B0CH4VCD6R</t>
+  </si>
+  <si>
+    <t>B0DFMKY4TT</t>
+  </si>
+  <si>
+    <t>FBA79835</t>
+  </si>
+  <si>
+    <t>B0FJ8TWCQZ</t>
+  </si>
+  <si>
+    <t>PB-06</t>
+  </si>
+  <si>
+    <t>FBA79836</t>
+  </si>
+  <si>
+    <t>B0FJ8Z1W81</t>
+  </si>
+  <si>
+    <t>PB-07</t>
+  </si>
+  <si>
+    <t>FBA79996</t>
+  </si>
+  <si>
+    <t>B0GW8Z556N</t>
+  </si>
+  <si>
+    <t>AM-C49</t>
+  </si>
+  <si>
+    <t>ELEGANT OFFICE SYSTEMS</t>
+  </si>
+  <si>
+    <t>B0CX1XK5R6</t>
+  </si>
+  <si>
+    <t>FBA79972</t>
+  </si>
+  <si>
+    <t>B0GCP1J2HC</t>
+  </si>
+  <si>
+    <t>M8</t>
+  </si>
+  <si>
+    <t>FBA80084</t>
+  </si>
+  <si>
+    <t>B0GXP97CZG</t>
+  </si>
+  <si>
+    <t>BE-4</t>
+  </si>
+  <si>
+    <t>FBA80012</t>
+  </si>
+  <si>
+    <t>B0GTZJF142</t>
+  </si>
+  <si>
+    <t>AM-Pro24</t>
+  </si>
+  <si>
+    <t>VMVCUBE INFOSYSTEM INDIA PRIVAT</t>
+  </si>
+  <si>
+    <t>THE SOUND PLAANET</t>
+  </si>
+  <si>
+    <t>B0B4KC7VBM</t>
+  </si>
+  <si>
+    <t>FBA79654</t>
+  </si>
+  <si>
+    <t>B0DN6MNS1X</t>
+  </si>
+  <si>
+    <t>AM-C11 Pro</t>
+  </si>
+  <si>
+    <t>FBA79959</t>
+  </si>
+  <si>
+    <t>B0G39ZHDYP</t>
+  </si>
+  <si>
+    <t>AM-W47 Wired</t>
+  </si>
+  <si>
+    <t>FBA80142</t>
+  </si>
+  <si>
+    <t>B0H3LHF2WW</t>
+  </si>
+  <si>
+    <t>AM-C5 White</t>
+  </si>
+  <si>
+    <t>B0B4G5JG4P</t>
+  </si>
+  <si>
+    <t>B0DFMLS8JG</t>
+  </si>
+  <si>
+    <t>FBA80002</t>
+  </si>
+  <si>
+    <t>B0GW96SHSK</t>
+  </si>
+  <si>
+    <t>AM-W33 Pro</t>
+  </si>
+  <si>
+    <t>B0CM9KJZWQ</t>
+  </si>
+  <si>
+    <t>FBA80003</t>
+  </si>
+  <si>
+    <t>B0GW92TTMS</t>
+  </si>
+  <si>
+    <t>AM-W32 Pro</t>
+  </si>
+  <si>
+    <t>FBA80110</t>
+  </si>
+  <si>
+    <t>B0H2Z6R6V8</t>
+  </si>
+  <si>
+    <t>X5</t>
+  </si>
+  <si>
+    <t>FBA80109</t>
+  </si>
+  <si>
+    <t>B0H2ZCQFTZ</t>
+  </si>
+  <si>
+    <t>M5</t>
+  </si>
+  <si>
+    <t>Charvi creators (Black Horse)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -728,6 +824,16 @@
       <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
     </font>
   </fonts>
   <fills count="6">
@@ -841,7 +947,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -901,9 +1007,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -921,6 +1024,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2635,7 +2747,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
-  <dimension ref="A1:AA688"/>
+  <dimension ref="A1:AA656"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -2691,19 +2803,19 @@
     </row>
     <row r="2" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
-        <v>80</v>
+        <v>21</v>
       </c>
       <c r="B2" s="18" t="s">
-        <v>81</v>
+        <v>23</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>82</v>
+        <v>22</v>
       </c>
       <c r="D2" s="7">
         <v>1</v>
       </c>
       <c r="E2" s="7">
-        <v>2881</v>
+        <v>1081</v>
       </c>
       <c r="F2" s="19" t="s">
         <v>33</v>
@@ -2714,19 +2826,19 @@
     </row>
     <row r="3" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="D3" s="7">
         <v>1</v>
       </c>
       <c r="E3" s="7">
-        <v>1801</v>
+        <v>2881</v>
       </c>
       <c r="F3" s="19" t="s">
         <v>33</v>
@@ -2736,726 +2848,1210 @@
       </c>
     </row>
     <row r="4" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="7" t="s">
-        <v>87</v>
+      <c r="A4" s="27" t="s">
+        <v>140</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>88</v>
-      </c>
-      <c r="C4" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="C4" s="27" t="s">
+        <v>174</v>
+      </c>
+      <c r="D4" s="27">
+        <v>1</v>
+      </c>
+      <c r="E4" s="7">
+        <v>720</v>
+      </c>
+      <c r="F4" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" s="18" t="s">
         <v>89</v>
-      </c>
-      <c r="D4" s="7">
-        <v>2</v>
-      </c>
-      <c r="E4" s="7">
-        <v>2881</v>
-      </c>
-      <c r="F4" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="G4" s="18" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D5" s="7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E5" s="7">
-        <v>5080</v>
+        <v>2542</v>
       </c>
       <c r="F5" s="19" t="s">
         <v>33</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>91</v>
+        <v>188</v>
       </c>
     </row>
     <row r="6" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D6" s="7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E6" s="7">
-        <v>4674</v>
+        <v>9254.24</v>
       </c>
       <c r="F6" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="18" t="s">
-        <v>91</v>
+      <c r="G6" s="20" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="7" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
-        <v>95</v>
+        <v>140</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>96</v>
+        <v>187</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>97</v>
+        <v>174</v>
       </c>
       <c r="D7" s="7">
-        <v>25</v>
-      </c>
-      <c r="E7" s="7">
-        <v>65250</v>
+        <v>10</v>
+      </c>
+      <c r="E7" s="8">
+        <v>6525.42</v>
       </c>
       <c r="F7" s="19" t="s">
         <v>33</v>
       </c>
       <c r="G7" s="20" t="s">
-        <v>98</v>
+        <v>189</v>
       </c>
     </row>
     <row r="8" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
-        <v>92</v>
+        <v>146</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>93</v>
+        <v>190</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>94</v>
+        <v>180</v>
       </c>
       <c r="D8" s="7">
-        <v>25</v>
-      </c>
-      <c r="E8" s="7">
-        <v>38550</v>
+        <v>2</v>
+      </c>
+      <c r="E8" s="8">
+        <v>4745.76</v>
       </c>
       <c r="F8" s="19" t="s">
         <v>33</v>
       </c>
       <c r="G8" s="20" t="s">
-        <v>98</v>
+        <v>189</v>
       </c>
     </row>
     <row r="9" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
-        <v>99</v>
+        <v>145</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>100</v>
+        <v>191</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>101</v>
+        <v>179</v>
       </c>
       <c r="D9" s="7">
-        <v>25</v>
-      </c>
-      <c r="E9" s="7">
-        <v>37075</v>
+        <v>2</v>
+      </c>
+      <c r="E9" s="8">
+        <v>2491.5300000000002</v>
       </c>
       <c r="F9" s="19" t="s">
         <v>33</v>
       </c>
       <c r="G9" s="20" t="s">
-        <v>98</v>
+        <v>189</v>
       </c>
     </row>
     <row r="10" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
-        <v>102</v>
+        <v>7</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>103</v>
+        <v>8</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>104</v>
+        <v>52</v>
       </c>
       <c r="D10" s="7">
-        <v>25</v>
-      </c>
-      <c r="E10" s="7">
-        <v>111225</v>
+        <v>10</v>
+      </c>
+      <c r="E10" s="8">
+        <v>29661.02</v>
       </c>
       <c r="F10" s="19" t="s">
         <v>33</v>
       </c>
       <c r="G10" s="20" t="s">
-        <v>98</v>
+        <v>189</v>
       </c>
     </row>
     <row r="11" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>11</v>
+        <v>192</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>10</v>
+        <v>157</v>
       </c>
       <c r="D11" s="7">
-        <v>5</v>
-      </c>
-      <c r="E11" s="7">
-        <v>8305</v>
+        <v>3</v>
+      </c>
+      <c r="E11" s="8">
+        <v>4271.1899999999996</v>
       </c>
       <c r="F11" s="19" t="s">
         <v>33</v>
       </c>
       <c r="G11" s="20" t="s">
-        <v>105</v>
+        <v>189</v>
       </c>
     </row>
     <row r="12" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
-        <v>106</v>
+        <v>53</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>108</v>
+        <v>55</v>
       </c>
       <c r="D12" s="7">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E12" s="8">
-        <v>17280</v>
+        <v>4449.1499999999996</v>
       </c>
       <c r="F12" s="19" t="s">
         <v>33</v>
       </c>
       <c r="G12" s="20" t="s">
-        <v>109</v>
+        <v>189</v>
       </c>
     </row>
     <row r="13" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
-        <v>12</v>
+        <v>43</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>14</v>
+        <v>193</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>13</v>
+        <v>44</v>
       </c>
       <c r="D13" s="7">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E13" s="8">
-        <v>17406.75</v>
+        <v>3440.68</v>
       </c>
       <c r="F13" s="19" t="s">
         <v>33</v>
       </c>
       <c r="G13" s="20" t="s">
-        <v>110</v>
+        <v>189</v>
       </c>
     </row>
     <row r="14" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
-        <v>111</v>
+        <v>136</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>112</v>
+        <v>194</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>113</v>
+        <v>170</v>
       </c>
       <c r="D14" s="7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E14" s="8">
-        <v>25087.88</v>
+        <v>4271.1899999999996</v>
       </c>
       <c r="F14" s="19" t="s">
         <v>33</v>
       </c>
       <c r="G14" s="20" t="s">
-        <v>114</v>
+        <v>189</v>
       </c>
     </row>
     <row r="15" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
-        <v>115</v>
+        <v>195</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>116</v>
+        <v>196</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>117</v>
+        <v>197</v>
       </c>
       <c r="D15" s="7">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E15" s="8">
-        <v>23713.98</v>
+        <v>11745.76</v>
       </c>
       <c r="F15" s="19" t="s">
         <v>33</v>
       </c>
       <c r="G15" s="20" t="s">
-        <v>114</v>
+        <v>189</v>
       </c>
     </row>
     <row r="16" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
-        <v>53</v>
+        <v>198</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>54</v>
+        <v>199</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>55</v>
+        <v>200</v>
       </c>
       <c r="D16" s="7">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E16" s="8">
-        <v>37061.440000000002</v>
+        <v>10203.39</v>
       </c>
       <c r="F16" s="19" t="s">
         <v>33</v>
       </c>
       <c r="G16" s="20" t="s">
-        <v>114</v>
+        <v>189</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>25</v>
+        <v>112</v>
       </c>
       <c r="D17" s="7">
         <v>5</v>
       </c>
-      <c r="E17" s="8">
-        <v>25197.03</v>
+      <c r="E17" s="7">
+        <v>4152.54</v>
       </c>
       <c r="F17" s="19" t="s">
         <v>33</v>
       </c>
       <c r="G17" s="20" t="s">
-        <v>114</v>
+        <v>189</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
-        <v>80</v>
+        <v>113</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>81</v>
+        <v>114</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>82</v>
+        <v>115</v>
       </c>
       <c r="D18" s="7">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E18" s="8">
-        <v>8184.07</v>
+        <v>5932.2</v>
       </c>
       <c r="F18" s="19" t="s">
         <v>33</v>
       </c>
       <c r="G18" s="20" t="s">
-        <v>114</v>
+        <v>189</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
-        <v>15</v>
+        <v>116</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>17</v>
+        <v>117</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>16</v>
+        <v>118</v>
       </c>
       <c r="D19" s="7">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E19" s="8">
-        <v>8065.42</v>
+        <v>5932.2</v>
       </c>
       <c r="F19" s="19" t="s">
         <v>33</v>
       </c>
       <c r="G19" s="20" t="s">
-        <v>114</v>
+        <v>189</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="s">
-        <v>118</v>
+        <v>201</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>119</v>
+        <v>202</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>79</v>
+        <v>203</v>
       </c>
       <c r="D20" s="7">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E20" s="8">
-        <v>48925.85</v>
+        <v>5338.98</v>
       </c>
       <c r="F20" s="19" t="s">
         <v>33</v>
       </c>
       <c r="G20" s="20" t="s">
-        <v>114</v>
+        <v>189</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="7" t="s">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="D21" s="7">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E21" s="8">
-        <v>23105.93</v>
+        <v>9966.1</v>
       </c>
       <c r="F21" s="19" t="s">
         <v>33</v>
       </c>
       <c r="G21" s="20" t="s">
-        <v>114</v>
+        <v>204</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="7" t="s">
-        <v>102</v>
+        <v>7</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>103</v>
+        <v>8</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>104</v>
+        <v>52</v>
       </c>
       <c r="D22" s="7">
-        <v>1</v>
-      </c>
-      <c r="E22" s="7">
-        <v>4151.95</v>
+        <v>6</v>
+      </c>
+      <c r="E22" s="8">
+        <v>17796.61</v>
       </c>
       <c r="F22" s="19" t="s">
         <v>33</v>
       </c>
       <c r="G22" s="20" t="s">
-        <v>114</v>
+        <v>204</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
-        <v>120</v>
+        <v>147</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>121</v>
+        <v>205</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>122</v>
+        <v>181</v>
       </c>
       <c r="D23" s="7">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E23" s="8">
-        <v>2965.51</v>
+        <v>17796.61</v>
       </c>
       <c r="F23" s="19" t="s">
         <v>33</v>
       </c>
       <c r="G23" s="20" t="s">
-        <v>114</v>
+        <v>204</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="7" t="s">
-        <v>123</v>
+        <v>21</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>124</v>
+        <v>23</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>125</v>
+        <v>22</v>
       </c>
       <c r="D24" s="7">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E24" s="8">
-        <v>4448.5600000000004</v>
+        <v>4271.1899999999996</v>
       </c>
       <c r="F24" s="19" t="s">
         <v>33</v>
       </c>
       <c r="G24" s="20" t="s">
-        <v>114</v>
+        <v>204</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="7" t="s">
-        <v>126</v>
+        <v>206</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>127</v>
+        <v>207</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>128</v>
+        <v>208</v>
       </c>
       <c r="D25" s="7">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E25" s="8">
-        <v>2668.9</v>
+        <v>50423.73</v>
       </c>
       <c r="F25" s="19" t="s">
         <v>33</v>
       </c>
       <c r="G25" s="20" t="s">
-        <v>114</v>
+        <v>204</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="7" t="s">
-        <v>129</v>
+        <v>209</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>130</v>
+        <v>210</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>131</v>
+        <v>211</v>
       </c>
       <c r="D26" s="7">
+        <v>6</v>
+      </c>
+      <c r="E26" s="8">
+        <v>13521.86</v>
+      </c>
+      <c r="F26" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G26" s="20" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="B27" s="18" t="s">
+        <v>213</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="D27" s="7">
+        <v>2</v>
+      </c>
+      <c r="E27" s="8">
+        <v>68272</v>
+      </c>
+      <c r="F27" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G27" s="18" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="B28" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="D28" s="7">
+        <v>2</v>
+      </c>
+      <c r="E28" s="8">
+        <v>5930</v>
+      </c>
+      <c r="F28" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G28" s="18" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="B29" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="D29" s="7">
+        <v>4</v>
+      </c>
+      <c r="E29" s="8">
+        <v>5424</v>
+      </c>
+      <c r="F29" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G29" s="18" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D30" s="7">
+        <v>3</v>
+      </c>
+      <c r="E30" s="8">
+        <v>8427.9599999999991</v>
+      </c>
+      <c r="F30" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G30" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="B31" s="18" t="s">
+        <v>217</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="D31" s="7">
         <v>1</v>
       </c>
-      <c r="E26" s="8">
-        <v>4745.17</v>
-      </c>
-      <c r="F26" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="G26" s="20" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="B27" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="C27" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="D27" s="21">
+      <c r="E31" s="8">
+        <v>1432.2</v>
+      </c>
+      <c r="F31" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G31" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B32" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D32" s="7">
         <v>1</v>
       </c>
-      <c r="E27" s="8">
-        <v>3114.47</v>
-      </c>
-      <c r="F27" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="G27" s="18" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="21" t="s">
+      <c r="E32" s="8">
+        <v>1983.05</v>
+      </c>
+      <c r="F32" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G32" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B33" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D33" s="7">
+        <v>2</v>
+      </c>
+      <c r="E33" s="8">
+        <v>826.28</v>
+      </c>
+      <c r="F33" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G33" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="B34" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="D34" s="7">
+        <v>2</v>
+      </c>
+      <c r="E34" s="8">
+        <v>3525.42</v>
+      </c>
+      <c r="F34" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G34" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="B35" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="D35" s="7">
+        <v>2</v>
+      </c>
+      <c r="E35" s="8">
+        <v>2313.56</v>
+      </c>
+      <c r="F35" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G35" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="B36" s="18" t="s">
+        <v>219</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="D36" s="7">
+        <v>5</v>
+      </c>
+      <c r="E36" s="8">
+        <v>14597.45</v>
+      </c>
+      <c r="F36" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G36" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B37" s="18" t="s">
+        <v>85</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="D37" s="7">
+        <v>15</v>
+      </c>
+      <c r="E37" s="8">
+        <v>19004.25</v>
+      </c>
+      <c r="F37" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G37" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="B38" s="18" t="s">
+        <v>190</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="D38" s="7">
+        <v>4</v>
+      </c>
+      <c r="E38" s="8">
+        <v>9033.8799999999992</v>
+      </c>
+      <c r="F38" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G38" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="B39" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="D39" s="7">
+        <v>4</v>
+      </c>
+      <c r="E39" s="8">
+        <v>20050.84</v>
+      </c>
+      <c r="F39" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G39" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="B40" s="18" t="s">
+        <v>222</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="D40" s="7">
+        <v>2</v>
+      </c>
+      <c r="E40" s="8">
+        <v>1432.2</v>
+      </c>
+      <c r="F40" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G40" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="B41" s="18" t="s">
+        <v>225</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="D41" s="7">
+        <v>1</v>
+      </c>
+      <c r="E41" s="8">
+        <v>1432.2</v>
+      </c>
+      <c r="F41" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G41" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="B42" s="18" t="s">
+        <v>191</v>
+      </c>
+      <c r="C42" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="D42" s="7">
+        <v>3</v>
+      </c>
+      <c r="E42" s="8">
+        <v>3800.85</v>
+      </c>
+      <c r="F42" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G42" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="B43" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="D43" s="7">
+        <v>5</v>
+      </c>
+      <c r="E43" s="8">
+        <v>10741.55</v>
+      </c>
+      <c r="F43" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G43" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="B44" s="18" t="s">
+        <v>227</v>
+      </c>
+      <c r="C44" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="D44" s="7">
+        <v>4</v>
+      </c>
+      <c r="E44" s="8">
+        <v>14101.68</v>
+      </c>
+      <c r="F44" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G44" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B45" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D45" s="7">
+        <v>5</v>
+      </c>
+      <c r="E45" s="7">
+        <v>5508.45</v>
+      </c>
+      <c r="F45" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G45" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="B46" s="18" t="s">
+        <v>228</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="D46" s="7">
+        <v>10</v>
+      </c>
+      <c r="E46" s="7">
+        <v>22584.7</v>
+      </c>
+      <c r="F46" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G46" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="B47" s="18" t="s">
+        <v>230</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="D47" s="7">
+        <v>4</v>
+      </c>
+      <c r="E47" s="7">
+        <v>7711.88</v>
+      </c>
+      <c r="F47" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G47" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="B48" s="18" t="s">
+        <v>232</v>
+      </c>
+      <c r="C48" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="D48" s="7">
+        <v>3</v>
+      </c>
+      <c r="E48" s="7">
+        <v>7932.21</v>
+      </c>
+      <c r="F48" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G48" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="B49" s="18" t="s">
+        <v>234</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="D49" s="7">
+        <v>2</v>
+      </c>
+      <c r="E49" s="7">
+        <v>6169.5</v>
+      </c>
+      <c r="F49" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G49" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="B50" s="18" t="s">
+        <v>237</v>
+      </c>
+      <c r="C50" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="D50" s="7">
+        <v>2</v>
+      </c>
+      <c r="E50" s="8">
+        <v>22144.06</v>
+      </c>
+      <c r="F50" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G50" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="B51" s="18" t="s">
+        <v>240</v>
+      </c>
+      <c r="C51" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="D51" s="7">
+        <v>4</v>
+      </c>
+      <c r="E51" s="8">
+        <v>44288.12</v>
+      </c>
+      <c r="F51" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G51" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B28" s="18" t="s">
+      <c r="B52" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="C28" s="21" t="s">
+      <c r="C52" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D28" s="21">
-        <v>1</v>
-      </c>
-      <c r="E28" s="8">
-        <v>3241.53</v>
-      </c>
-      <c r="F28" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="G28" s="18" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="21" t="s">
-        <v>56</v>
-      </c>
-      <c r="B29" s="18" t="s">
-        <v>57</v>
-      </c>
-      <c r="C29" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="D29" s="21">
-        <v>1</v>
-      </c>
-      <c r="E29" s="8">
-        <v>1970.34</v>
-      </c>
-      <c r="F29" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="G29" s="18" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="21" t="s">
-        <v>133</v>
-      </c>
-      <c r="B30" s="18" t="s">
-        <v>134</v>
-      </c>
-      <c r="C30" s="21" t="s">
-        <v>135</v>
-      </c>
-      <c r="D30" s="21">
+      <c r="D52" s="7">
         <v>2</v>
       </c>
-      <c r="E30" s="8">
-        <v>11440.68</v>
-      </c>
-      <c r="F30" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="G30" s="18" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="B31" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="C31" s="21" t="s">
-        <v>136</v>
-      </c>
-      <c r="D31" s="21">
-        <v>4</v>
-      </c>
-      <c r="E31" s="8">
-        <v>3559.32</v>
-      </c>
-      <c r="F31" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="G31" s="18" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="21" t="s">
-        <v>137</v>
-      </c>
-      <c r="B32" s="18" t="s">
-        <v>138</v>
-      </c>
-      <c r="C32" s="21" t="s">
-        <v>139</v>
-      </c>
-      <c r="D32" s="21">
+      <c r="E52" s="8">
+        <v>6059.32</v>
+      </c>
+      <c r="F52" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G52" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="B53" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="C53" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="D53" s="7">
+        <v>10</v>
+      </c>
+      <c r="E53" s="8">
+        <v>47372.9</v>
+      </c>
+      <c r="F53" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G53" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B54" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="C54" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="D54" s="7">
+        <v>10</v>
+      </c>
+      <c r="E54" s="8">
+        <v>45444.9</v>
+      </c>
+      <c r="F54" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G54" s="18" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="B55" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="C55" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="D55" s="29">
         <v>2</v>
       </c>
-      <c r="E32" s="8">
-        <v>2542.38</v>
-      </c>
-      <c r="F32" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="G32" s="18" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="21" t="s">
-        <v>140</v>
-      </c>
-      <c r="B33" s="18" t="s">
-        <v>141</v>
-      </c>
-      <c r="C33" s="21" t="s">
-        <v>142</v>
-      </c>
-      <c r="D33" s="21">
-        <v>2</v>
-      </c>
-      <c r="E33" s="8">
-        <v>2542.38</v>
-      </c>
-      <c r="F33" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="G33" s="18" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="35" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="36" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="37" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="38" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="39" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="40" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="41" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="42" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="43" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="44" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="45" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="46" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="47" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="48" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="49" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="50" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="51" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="52" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="53" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="54" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="55" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="56" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="57" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="58" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="59" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="60" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="61" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="62" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="63" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="64" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+      <c r="E55" s="8">
+        <v>2978</v>
+      </c>
+      <c r="F55" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="G55" s="18" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="57" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="58" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="59" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="60" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="61" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="62" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="63" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="64" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="65" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="66" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="67" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -4048,38 +4644,6 @@
     <row r="654" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="655" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="656" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="657" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="658" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="659" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="660" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="661" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="662" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="663" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="664" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="665" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="666" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="667" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="668" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="669" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="670" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="671" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="672" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="673" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="674" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="675" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="676" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="677" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="678" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="679" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="680" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="681" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="682" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="683" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="684" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="685" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="686" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="687" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="688" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -4094,37 +4658,37 @@
     <col min="1" max="1" width="14.5546875" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
     <col min="3" max="3" width="14.109375" customWidth="1"/>
-    <col min="4" max="4" width="17.77734375" style="27" customWidth="1"/>
+    <col min="4" max="4" width="17.77734375" style="26" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="22" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="22" t="s">
+      <c r="A1" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="22" t="s">
+      <c r="C1" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="23" t="s">
+      <c r="D1" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="22" t="s">
+      <c r="E1" s="21" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="C2" s="25">
+      <c r="C2" s="24">
         <v>13</v>
       </c>
-      <c r="D2" s="26">
+      <c r="D2" s="25">
         <v>52504.237288135599</v>
       </c>
       <c r="E2" t="s">
@@ -4132,16 +4696,16 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="24" t="s">
+      <c r="A3" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="24" t="s">
+      <c r="B3" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="25">
+      <c r="C3" s="24">
         <v>14</v>
       </c>
-      <c r="D3" s="26">
+      <c r="D3" s="25">
         <v>30853.389830508477</v>
       </c>
       <c r="E3" t="s">
@@ -4149,917 +4713,917 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="24" t="s">
+      <c r="A4" s="23" t="s">
+        <v>119</v>
+      </c>
+      <c r="B4" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="C4" s="24">
+        <v>2</v>
+      </c>
+      <c r="D4" s="25">
+        <v>7308.4745762711864</v>
+      </c>
+      <c r="E4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="B5" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="24">
+        <v>5</v>
+      </c>
+      <c r="D5" s="25">
+        <v>6294.0677966101703</v>
+      </c>
+      <c r="E5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="23" t="s">
+        <v>104</v>
+      </c>
+      <c r="B6" s="23" t="s">
+        <v>105</v>
+      </c>
+      <c r="C6" s="24">
+        <v>5</v>
+      </c>
+      <c r="D6" s="25">
+        <v>6265.2542372881362</v>
+      </c>
+      <c r="E6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="23" t="s">
+        <v>120</v>
+      </c>
+      <c r="B7" s="23" t="s">
+        <v>154</v>
+      </c>
+      <c r="C7" s="24">
+        <v>2</v>
+      </c>
+      <c r="D7" s="25">
+        <v>5749.1525423728817</v>
+      </c>
+      <c r="E7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="23" t="s">
+        <v>121</v>
+      </c>
+      <c r="B8" s="23" t="s">
+        <v>155</v>
+      </c>
+      <c r="C8" s="24">
+        <v>1</v>
+      </c>
+      <c r="D8" s="25">
+        <v>5116.1016949152545</v>
+      </c>
+      <c r="E8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="23" t="s">
+        <v>122</v>
+      </c>
+      <c r="B9" s="23" t="s">
+        <v>156</v>
+      </c>
+      <c r="C9" s="24">
+        <v>1</v>
+      </c>
+      <c r="D9" s="25">
+        <v>4861.8644067796613</v>
+      </c>
+      <c r="E9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="23" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="24">
+        <v>1</v>
+      </c>
+      <c r="D10" s="25">
+        <v>3888.9830508474579</v>
+      </c>
+      <c r="E10" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="23" t="s">
+        <v>123</v>
+      </c>
+      <c r="B11" s="23" t="s">
+        <v>157</v>
+      </c>
+      <c r="C11" s="24">
+        <v>2</v>
+      </c>
+      <c r="D11" s="25">
+        <v>3838.9830508474579</v>
+      </c>
+      <c r="E11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="23" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="24">
+        <v>2</v>
+      </c>
+      <c r="D12" s="25">
+        <v>3816.9491525423732</v>
+      </c>
+      <c r="E12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="23" t="s">
+        <v>124</v>
+      </c>
+      <c r="B13" s="23" t="s">
+        <v>158</v>
+      </c>
+      <c r="C13" s="24">
+        <v>2</v>
+      </c>
+      <c r="D13" s="25">
+        <v>3191.5254237288136</v>
+      </c>
+      <c r="E13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="B14" s="23" t="s">
+        <v>159</v>
+      </c>
+      <c r="C14" s="24">
+        <v>1</v>
+      </c>
+      <c r="D14" s="25">
+        <v>3166.1016949152545</v>
+      </c>
+      <c r="E14" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="23" t="s">
+        <v>126</v>
+      </c>
+      <c r="B15" s="23" t="s">
+        <v>160</v>
+      </c>
+      <c r="C15" s="24">
+        <v>1</v>
+      </c>
+      <c r="D15" s="25">
+        <v>3066.1016949152545</v>
+      </c>
+      <c r="E15" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="23" t="s">
+        <v>93</v>
+      </c>
+      <c r="B16" s="23" t="s">
+        <v>95</v>
+      </c>
+      <c r="C16" s="24">
+        <v>1</v>
+      </c>
+      <c r="D16" s="25">
+        <v>2917.7966101694915</v>
+      </c>
+      <c r="E16" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="23" t="s">
+        <v>127</v>
+      </c>
+      <c r="B17" s="23" t="s">
+        <v>161</v>
+      </c>
+      <c r="C17" s="24">
+        <v>1</v>
+      </c>
+      <c r="D17" s="25">
+        <v>2907.6271186440681</v>
+      </c>
+      <c r="E17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="24">
+        <v>1</v>
+      </c>
+      <c r="D18" s="25">
+        <v>2888.1355932203392</v>
+      </c>
+      <c r="E18" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="B19" s="23" t="s">
+        <v>82</v>
+      </c>
+      <c r="C19" s="24">
+        <v>1</v>
+      </c>
+      <c r="D19" s="25">
+        <v>2638.9830508474579</v>
+      </c>
+      <c r="E19" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="23" t="s">
+        <v>53</v>
+      </c>
+      <c r="B20" s="23" t="s">
+        <v>55</v>
+      </c>
+      <c r="C20" s="24">
+        <v>1</v>
+      </c>
+      <c r="D20" s="25">
+        <v>1938.9830508474577</v>
+      </c>
+      <c r="E20" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="23" t="s">
+        <v>128</v>
+      </c>
+      <c r="B21" s="23" t="s">
+        <v>162</v>
+      </c>
+      <c r="C21" s="24">
+        <v>1</v>
+      </c>
+      <c r="D21" s="25">
+        <v>1599.1525423728815</v>
+      </c>
+      <c r="E21" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="B22" s="23" t="s">
+        <v>88</v>
+      </c>
+      <c r="C22" s="24">
+        <v>1</v>
+      </c>
+      <c r="D22" s="25">
+        <v>1206.7796610169491</v>
+      </c>
+      <c r="E22" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="B23" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="C23" s="24">
+        <v>2</v>
+      </c>
+      <c r="D23" s="25">
+        <v>1125.4237288135594</v>
+      </c>
+      <c r="E23" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" s="23" t="s">
+        <v>129</v>
+      </c>
+      <c r="B24" s="23" t="s">
+        <v>163</v>
+      </c>
+      <c r="C24" s="24">
+        <v>1</v>
+      </c>
+      <c r="D24" s="25">
+        <v>683.05084745762713</v>
+      </c>
+      <c r="E24" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" s="23" t="s">
+        <v>130</v>
+      </c>
+      <c r="B25" s="23" t="s">
+        <v>164</v>
+      </c>
+      <c r="C25" s="24">
+        <v>0</v>
+      </c>
+      <c r="D25" s="25">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" s="23" t="s">
+        <v>131</v>
+      </c>
+      <c r="B26" s="23" t="s">
+        <v>165</v>
+      </c>
+      <c r="C26" s="24">
+        <v>0</v>
+      </c>
+      <c r="D26" s="25">
+        <v>0</v>
+      </c>
+      <c r="E26" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" s="23" t="s">
+        <v>132</v>
+      </c>
+      <c r="B27" s="23" t="s">
+        <v>166</v>
+      </c>
+      <c r="C27" s="24">
+        <v>0</v>
+      </c>
+      <c r="D27" s="25">
+        <v>0</v>
+      </c>
+      <c r="E27" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" s="23" t="s">
+        <v>84</v>
+      </c>
+      <c r="B28" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="C28" s="24">
+        <v>0</v>
+      </c>
+      <c r="D28" s="25">
+        <v>0</v>
+      </c>
+      <c r="E28" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" s="23" t="s">
+        <v>133</v>
+      </c>
+      <c r="B29" s="23" t="s">
+        <v>167</v>
+      </c>
+      <c r="C29" s="24">
+        <v>0</v>
+      </c>
+      <c r="D29" s="25">
+        <v>0</v>
+      </c>
+      <c r="E29" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" s="23" t="s">
+        <v>27</v>
+      </c>
+      <c r="B30" s="23" t="s">
+        <v>28</v>
+      </c>
+      <c r="C30" s="24">
+        <v>0</v>
+      </c>
+      <c r="D30" s="25">
+        <v>0</v>
+      </c>
+      <c r="E30" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" s="23" t="s">
+        <v>56</v>
+      </c>
+      <c r="B31" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="C31" s="24">
+        <v>0</v>
+      </c>
+      <c r="D31" s="25">
+        <v>0</v>
+      </c>
+      <c r="E31" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" s="23" t="s">
+        <v>134</v>
+      </c>
+      <c r="B32" s="23" t="s">
+        <v>168</v>
+      </c>
+      <c r="C32" s="24">
+        <v>0</v>
+      </c>
+      <c r="D32" s="25">
+        <v>0</v>
+      </c>
+      <c r="E32" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="B33" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="C33" s="24">
+        <v>0</v>
+      </c>
+      <c r="D33" s="25">
+        <v>0</v>
+      </c>
+      <c r="E33" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A34" s="23" t="s">
+        <v>135</v>
+      </c>
+      <c r="B34" s="23" t="s">
+        <v>169</v>
+      </c>
+      <c r="C34" s="24">
+        <v>0</v>
+      </c>
+      <c r="D34" s="25">
+        <v>0</v>
+      </c>
+      <c r="E34" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A35" s="23" t="s">
+        <v>136</v>
+      </c>
+      <c r="B35" s="23" t="s">
+        <v>170</v>
+      </c>
+      <c r="C35" s="24">
+        <v>0</v>
+      </c>
+      <c r="D35" s="25">
+        <v>0</v>
+      </c>
+      <c r="E35" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" s="23" t="s">
+        <v>137</v>
+      </c>
+      <c r="B36" s="23" t="s">
+        <v>171</v>
+      </c>
+      <c r="C36" s="24">
+        <v>0</v>
+      </c>
+      <c r="D36" s="25">
+        <v>0</v>
+      </c>
+      <c r="E36" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" s="23" t="s">
+        <v>138</v>
+      </c>
+      <c r="B37" s="23" t="s">
+        <v>172</v>
+      </c>
+      <c r="C37" s="24">
+        <v>0</v>
+      </c>
+      <c r="D37" s="25">
+        <v>0</v>
+      </c>
+      <c r="E37" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="B38" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="C38" s="24">
+        <v>0</v>
+      </c>
+      <c r="D38" s="25">
+        <v>0</v>
+      </c>
+      <c r="E38" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" s="23" t="s">
+        <v>139</v>
+      </c>
+      <c r="B39" s="23" t="s">
+        <v>173</v>
+      </c>
+      <c r="C39" s="24">
+        <v>0</v>
+      </c>
+      <c r="D39" s="25">
+        <v>0</v>
+      </c>
+      <c r="E39" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" s="23" t="s">
+        <v>140</v>
+      </c>
+      <c r="B40" s="23" t="s">
+        <v>174</v>
+      </c>
+      <c r="C40" s="24">
+        <v>0</v>
+      </c>
+      <c r="D40" s="25">
+        <v>0</v>
+      </c>
+      <c r="E40" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="B41" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="C41" s="24">
+        <v>0</v>
+      </c>
+      <c r="D41" s="25">
+        <v>0</v>
+      </c>
+      <c r="E41" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="B42" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="C42" s="24">
+        <v>0</v>
+      </c>
+      <c r="D42" s="25">
+        <v>0</v>
+      </c>
+      <c r="E42" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" s="23" t="s">
+        <v>141</v>
+      </c>
+      <c r="B43" s="23" t="s">
+        <v>175</v>
+      </c>
+      <c r="C43" s="24">
+        <v>0</v>
+      </c>
+      <c r="D43" s="25">
+        <v>0</v>
+      </c>
+      <c r="E43" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44" s="23" t="s">
+        <v>142</v>
+      </c>
+      <c r="B44" s="23" t="s">
+        <v>176</v>
+      </c>
+      <c r="C44" s="24">
+        <v>0</v>
+      </c>
+      <c r="D44" s="25">
+        <v>0</v>
+      </c>
+      <c r="E44" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="B45" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="C45" s="24">
+        <v>0</v>
+      </c>
+      <c r="D45" s="25">
+        <v>0</v>
+      </c>
+      <c r="E45" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A46" s="23" t="s">
         <v>143</v>
       </c>
-      <c r="B4" s="24" t="s">
+      <c r="B46" s="23" t="s">
         <v>177</v>
       </c>
-      <c r="C4" s="25">
-        <v>2</v>
-      </c>
-      <c r="D4" s="26">
-        <v>7308.4745762711864</v>
-      </c>
-      <c r="E4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="B5" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="C5" s="25">
-        <v>5</v>
-      </c>
-      <c r="D5" s="26">
-        <v>6294.0677966101703</v>
-      </c>
-      <c r="E5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="24" t="s">
-        <v>115</v>
-      </c>
-      <c r="B6" s="24" t="s">
-        <v>117</v>
-      </c>
-      <c r="C6" s="25">
-        <v>5</v>
-      </c>
-      <c r="D6" s="26">
-        <v>6265.2542372881362</v>
-      </c>
-      <c r="E6" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="24" t="s">
+      <c r="C46" s="24">
+        <v>0</v>
+      </c>
+      <c r="D46" s="25">
+        <v>0</v>
+      </c>
+      <c r="E46" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A47" s="23" t="s">
         <v>144</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B47" s="23" t="s">
         <v>178</v>
       </c>
-      <c r="C7" s="25">
-        <v>2</v>
-      </c>
-      <c r="D7" s="26">
-        <v>5749.1525423728817</v>
-      </c>
-      <c r="E7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="24" t="s">
+      <c r="C47" s="24">
+        <v>0</v>
+      </c>
+      <c r="D47" s="25">
+        <v>0</v>
+      </c>
+      <c r="E47" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="B48" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="C48" s="24">
+        <v>0</v>
+      </c>
+      <c r="D48" s="25">
+        <v>0</v>
+      </c>
+      <c r="E48" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A49" s="23" t="s">
         <v>145</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="B49" s="23" t="s">
         <v>179</v>
       </c>
-      <c r="C8" s="25">
-        <v>1</v>
-      </c>
-      <c r="D8" s="26">
-        <v>5116.1016949152545</v>
-      </c>
-      <c r="E8" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="24" t="s">
+      <c r="C49" s="24">
+        <v>0</v>
+      </c>
+      <c r="D49" s="25">
+        <v>0</v>
+      </c>
+      <c r="E49" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50" s="23" t="s">
         <v>146</v>
       </c>
-      <c r="B9" s="24" t="s">
+      <c r="B50" s="23" t="s">
         <v>180</v>
       </c>
-      <c r="C9" s="25">
-        <v>1</v>
-      </c>
-      <c r="D9" s="26">
-        <v>4861.8644067796613</v>
-      </c>
-      <c r="E9" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="24" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10" s="25">
-        <v>1</v>
-      </c>
-      <c r="D10" s="26">
-        <v>3888.9830508474579</v>
-      </c>
-      <c r="E10" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="24" t="s">
+      <c r="C50" s="24">
+        <v>0</v>
+      </c>
+      <c r="D50" s="25">
+        <v>0</v>
+      </c>
+      <c r="E50" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="B51" s="23" t="s">
+        <v>25</v>
+      </c>
+      <c r="C51" s="24">
+        <v>0</v>
+      </c>
+      <c r="D51" s="25">
+        <v>0</v>
+      </c>
+      <c r="E51" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A52" s="23" t="s">
         <v>147</v>
       </c>
-      <c r="B11" s="24" t="s">
+      <c r="B52" s="23" t="s">
         <v>181</v>
       </c>
-      <c r="C11" s="25">
-        <v>2</v>
-      </c>
-      <c r="D11" s="26">
-        <v>3838.9830508474579</v>
-      </c>
-      <c r="E11" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="24" t="s">
-        <v>39</v>
-      </c>
-      <c r="B12" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" s="25">
-        <v>2</v>
-      </c>
-      <c r="D12" s="26">
-        <v>3816.9491525423732</v>
-      </c>
-      <c r="E12" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="24" t="s">
+      <c r="C52" s="24">
+        <v>0</v>
+      </c>
+      <c r="D52" s="25">
+        <v>0</v>
+      </c>
+      <c r="E52" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A53" s="23" t="s">
         <v>148</v>
       </c>
-      <c r="B13" s="24" t="s">
+      <c r="B53" s="23" t="s">
         <v>182</v>
       </c>
-      <c r="C13" s="25">
-        <v>2</v>
-      </c>
-      <c r="D13" s="26">
-        <v>3191.5254237288136</v>
-      </c>
-      <c r="E13" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="24" t="s">
+      <c r="C53" s="24">
+        <v>0</v>
+      </c>
+      <c r="D53" s="25">
+        <v>0</v>
+      </c>
+      <c r="E53" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A54" s="23" t="s">
         <v>149</v>
       </c>
-      <c r="B14" s="24" t="s">
+      <c r="B54" s="23" t="s">
         <v>183</v>
       </c>
-      <c r="C14" s="25">
-        <v>1</v>
-      </c>
-      <c r="D14" s="26">
-        <v>3166.1016949152545</v>
-      </c>
-      <c r="E14" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="24" t="s">
+      <c r="C54" s="24">
+        <v>0</v>
+      </c>
+      <c r="D54" s="25">
+        <v>0</v>
+      </c>
+      <c r="E54" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A55" s="23" t="s">
         <v>150</v>
       </c>
-      <c r="B15" s="24" t="s">
+      <c r="B55" s="23" t="s">
         <v>184</v>
       </c>
-      <c r="C15" s="25">
-        <v>1</v>
-      </c>
-      <c r="D15" s="26">
-        <v>3066.1016949152545</v>
-      </c>
-      <c r="E15" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="24" t="s">
-        <v>95</v>
-      </c>
-      <c r="B16" s="24" t="s">
-        <v>97</v>
-      </c>
-      <c r="C16" s="25">
-        <v>1</v>
-      </c>
-      <c r="D16" s="26">
-        <v>2917.7966101694915</v>
-      </c>
-      <c r="E16" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="24" t="s">
+      <c r="C55" s="24">
+        <v>0</v>
+      </c>
+      <c r="D55" s="25">
+        <v>0</v>
+      </c>
+      <c r="E55" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A56" s="23" t="s">
         <v>151</v>
       </c>
-      <c r="B17" s="24" t="s">
+      <c r="B56" s="23" t="s">
         <v>185</v>
       </c>
-      <c r="C17" s="25">
-        <v>1</v>
-      </c>
-      <c r="D17" s="26">
-        <v>2907.6271186440681</v>
-      </c>
-      <c r="E17" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="B18" s="24" t="s">
-        <v>16</v>
-      </c>
-      <c r="C18" s="25">
-        <v>1</v>
-      </c>
-      <c r="D18" s="26">
-        <v>2888.1355932203392</v>
-      </c>
-      <c r="E18" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="24" t="s">
-        <v>80</v>
-      </c>
-      <c r="B19" s="24" t="s">
-        <v>82</v>
-      </c>
-      <c r="C19" s="25">
-        <v>1</v>
-      </c>
-      <c r="D19" s="26">
-        <v>2638.9830508474579</v>
-      </c>
-      <c r="E19" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="24" t="s">
-        <v>53</v>
-      </c>
-      <c r="B20" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="C20" s="25">
-        <v>1</v>
-      </c>
-      <c r="D20" s="26">
-        <v>1938.9830508474577</v>
-      </c>
-      <c r="E20" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="24" t="s">
+      <c r="C56" s="24">
+        <v>0</v>
+      </c>
+      <c r="D56" s="25">
+        <v>0</v>
+      </c>
+      <c r="E56" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A57" s="23" t="s">
         <v>152</v>
       </c>
-      <c r="B21" s="24" t="s">
+      <c r="B57" s="23" t="s">
         <v>186</v>
       </c>
-      <c r="C21" s="25">
-        <v>1</v>
-      </c>
-      <c r="D21" s="26">
-        <v>1599.1525423728815</v>
-      </c>
-      <c r="E21" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" s="24" t="s">
-        <v>87</v>
-      </c>
-      <c r="B22" s="24" t="s">
-        <v>89</v>
-      </c>
-      <c r="C22" s="25">
-        <v>1</v>
-      </c>
-      <c r="D22" s="26">
-        <v>1206.7796610169491</v>
-      </c>
-      <c r="E22" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="24" t="s">
-        <v>49</v>
-      </c>
-      <c r="B23" s="24" t="s">
-        <v>51</v>
-      </c>
-      <c r="C23" s="25">
-        <v>2</v>
-      </c>
-      <c r="D23" s="26">
-        <v>1125.4237288135594</v>
-      </c>
-      <c r="E23" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" s="24" t="s">
-        <v>153</v>
-      </c>
-      <c r="B24" s="24" t="s">
-        <v>187</v>
-      </c>
-      <c r="C24" s="25">
-        <v>1</v>
-      </c>
-      <c r="D24" s="26">
-        <v>683.05084745762713</v>
-      </c>
-      <c r="E24" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" s="24" t="s">
-        <v>154</v>
-      </c>
-      <c r="B25" s="24" t="s">
-        <v>188</v>
-      </c>
-      <c r="C25" s="25">
-        <v>0</v>
-      </c>
-      <c r="D25" s="26">
-        <v>0</v>
-      </c>
-      <c r="E25" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A26" s="24" t="s">
-        <v>155</v>
-      </c>
-      <c r="B26" s="24" t="s">
-        <v>189</v>
-      </c>
-      <c r="C26" s="25">
-        <v>0</v>
-      </c>
-      <c r="D26" s="26">
-        <v>0</v>
-      </c>
-      <c r="E26" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A27" s="24" t="s">
-        <v>156</v>
-      </c>
-      <c r="B27" s="24" t="s">
-        <v>190</v>
-      </c>
-      <c r="C27" s="25">
-        <v>0</v>
-      </c>
-      <c r="D27" s="26">
-        <v>0</v>
-      </c>
-      <c r="E27" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A28" s="24" t="s">
-        <v>84</v>
-      </c>
-      <c r="B28" s="24" t="s">
-        <v>86</v>
-      </c>
-      <c r="C28" s="25">
-        <v>0</v>
-      </c>
-      <c r="D28" s="26">
-        <v>0</v>
-      </c>
-      <c r="E28" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A29" s="24" t="s">
-        <v>157</v>
-      </c>
-      <c r="B29" s="24" t="s">
-        <v>191</v>
-      </c>
-      <c r="C29" s="25">
-        <v>0</v>
-      </c>
-      <c r="D29" s="26">
-        <v>0</v>
-      </c>
-      <c r="E29" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A30" s="24" t="s">
-        <v>27</v>
-      </c>
-      <c r="B30" s="24" t="s">
-        <v>28</v>
-      </c>
-      <c r="C30" s="25">
-        <v>0</v>
-      </c>
-      <c r="D30" s="26">
-        <v>0</v>
-      </c>
-      <c r="E30" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A31" s="24" t="s">
-        <v>56</v>
-      </c>
-      <c r="B31" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="C31" s="25">
-        <v>0</v>
-      </c>
-      <c r="D31" s="26">
-        <v>0</v>
-      </c>
-      <c r="E31" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A32" s="24" t="s">
-        <v>158</v>
-      </c>
-      <c r="B32" s="24" t="s">
-        <v>192</v>
-      </c>
-      <c r="C32" s="25">
-        <v>0</v>
-      </c>
-      <c r="D32" s="26">
-        <v>0</v>
-      </c>
-      <c r="E32" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A33" s="24" t="s">
-        <v>43</v>
-      </c>
-      <c r="B33" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="C33" s="25">
-        <v>0</v>
-      </c>
-      <c r="D33" s="26">
-        <v>0</v>
-      </c>
-      <c r="E33" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A34" s="24" t="s">
-        <v>159</v>
-      </c>
-      <c r="B34" s="24" t="s">
-        <v>193</v>
-      </c>
-      <c r="C34" s="25">
-        <v>0</v>
-      </c>
-      <c r="D34" s="26">
-        <v>0</v>
-      </c>
-      <c r="E34" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A35" s="24" t="s">
-        <v>160</v>
-      </c>
-      <c r="B35" s="24" t="s">
-        <v>194</v>
-      </c>
-      <c r="C35" s="25">
-        <v>0</v>
-      </c>
-      <c r="D35" s="26">
-        <v>0</v>
-      </c>
-      <c r="E35" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A36" s="24" t="s">
-        <v>161</v>
-      </c>
-      <c r="B36" s="24" t="s">
-        <v>195</v>
-      </c>
-      <c r="C36" s="25">
-        <v>0</v>
-      </c>
-      <c r="D36" s="26">
-        <v>0</v>
-      </c>
-      <c r="E36" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A37" s="24" t="s">
-        <v>162</v>
-      </c>
-      <c r="B37" s="24" t="s">
-        <v>196</v>
-      </c>
-      <c r="C37" s="25">
-        <v>0</v>
-      </c>
-      <c r="D37" s="26">
-        <v>0</v>
-      </c>
-      <c r="E37" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A38" s="24" t="s">
-        <v>41</v>
-      </c>
-      <c r="B38" s="24" t="s">
-        <v>42</v>
-      </c>
-      <c r="C38" s="25">
-        <v>0</v>
-      </c>
-      <c r="D38" s="26">
-        <v>0</v>
-      </c>
-      <c r="E38" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A39" s="24" t="s">
-        <v>163</v>
-      </c>
-      <c r="B39" s="24" t="s">
-        <v>197</v>
-      </c>
-      <c r="C39" s="25">
-        <v>0</v>
-      </c>
-      <c r="D39" s="26">
-        <v>0</v>
-      </c>
-      <c r="E39" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A40" s="24" t="s">
-        <v>164</v>
-      </c>
-      <c r="B40" s="24" t="s">
-        <v>198</v>
-      </c>
-      <c r="C40" s="25">
-        <v>0</v>
-      </c>
-      <c r="D40" s="26">
-        <v>0</v>
-      </c>
-      <c r="E40" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A41" s="24" t="s">
-        <v>106</v>
-      </c>
-      <c r="B41" s="24" t="s">
-        <v>108</v>
-      </c>
-      <c r="C41" s="25">
-        <v>0</v>
-      </c>
-      <c r="D41" s="26">
-        <v>0</v>
-      </c>
-      <c r="E41" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A42" s="24" t="s">
-        <v>37</v>
-      </c>
-      <c r="B42" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="C42" s="25">
-        <v>0</v>
-      </c>
-      <c r="D42" s="26">
-        <v>0</v>
-      </c>
-      <c r="E42" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A43" s="24" t="s">
-        <v>165</v>
-      </c>
-      <c r="B43" s="24" t="s">
-        <v>199</v>
-      </c>
-      <c r="C43" s="25">
-        <v>0</v>
-      </c>
-      <c r="D43" s="26">
-        <v>0</v>
-      </c>
-      <c r="E43" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A44" s="24" t="s">
-        <v>166</v>
-      </c>
-      <c r="B44" s="24" t="s">
-        <v>200</v>
-      </c>
-      <c r="C44" s="25">
-        <v>0</v>
-      </c>
-      <c r="D44" s="26">
-        <v>0</v>
-      </c>
-      <c r="E44" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A45" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="B45" s="24" t="s">
-        <v>64</v>
-      </c>
-      <c r="C45" s="25">
-        <v>0</v>
-      </c>
-      <c r="D45" s="26">
-        <v>0</v>
-      </c>
-      <c r="E45" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A46" s="24" t="s">
-        <v>167</v>
-      </c>
-      <c r="B46" s="24" t="s">
-        <v>201</v>
-      </c>
-      <c r="C46" s="25">
-        <v>0</v>
-      </c>
-      <c r="D46" s="26">
-        <v>0</v>
-      </c>
-      <c r="E46" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A47" s="24" t="s">
-        <v>168</v>
-      </c>
-      <c r="B47" s="24" t="s">
-        <v>202</v>
-      </c>
-      <c r="C47" s="25">
-        <v>0</v>
-      </c>
-      <c r="D47" s="26">
-        <v>0</v>
-      </c>
-      <c r="E47" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A48" s="24" t="s">
-        <v>21</v>
-      </c>
-      <c r="B48" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="C48" s="25">
-        <v>0</v>
-      </c>
-      <c r="D48" s="26">
-        <v>0</v>
-      </c>
-      <c r="E48" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A49" s="24" t="s">
-        <v>169</v>
-      </c>
-      <c r="B49" s="24" t="s">
-        <v>203</v>
-      </c>
-      <c r="C49" s="25">
-        <v>0</v>
-      </c>
-      <c r="D49" s="26">
-        <v>0</v>
-      </c>
-      <c r="E49" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A50" s="24" t="s">
-        <v>170</v>
-      </c>
-      <c r="B50" s="24" t="s">
-        <v>204</v>
-      </c>
-      <c r="C50" s="25">
-        <v>0</v>
-      </c>
-      <c r="D50" s="26">
-        <v>0</v>
-      </c>
-      <c r="E50" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A51" s="24" t="s">
-        <v>24</v>
-      </c>
-      <c r="B51" s="24" t="s">
-        <v>25</v>
-      </c>
-      <c r="C51" s="25">
-        <v>0</v>
-      </c>
-      <c r="D51" s="26">
-        <v>0</v>
-      </c>
-      <c r="E51" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A52" s="24" t="s">
-        <v>171</v>
-      </c>
-      <c r="B52" s="24" t="s">
-        <v>205</v>
-      </c>
-      <c r="C52" s="25">
-        <v>0</v>
-      </c>
-      <c r="D52" s="26">
-        <v>0</v>
-      </c>
-      <c r="E52" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A53" s="24" t="s">
-        <v>172</v>
-      </c>
-      <c r="B53" s="24" t="s">
-        <v>206</v>
-      </c>
-      <c r="C53" s="25">
-        <v>0</v>
-      </c>
-      <c r="D53" s="26">
-        <v>0</v>
-      </c>
-      <c r="E53" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A54" s="24" t="s">
-        <v>173</v>
-      </c>
-      <c r="B54" s="24" t="s">
-        <v>207</v>
-      </c>
-      <c r="C54" s="25">
-        <v>0</v>
-      </c>
-      <c r="D54" s="26">
-        <v>0</v>
-      </c>
-      <c r="E54" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A55" s="24" t="s">
-        <v>174</v>
-      </c>
-      <c r="B55" s="24" t="s">
-        <v>208</v>
-      </c>
-      <c r="C55" s="25">
-        <v>0</v>
-      </c>
-      <c r="D55" s="26">
-        <v>0</v>
-      </c>
-      <c r="E55" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A56" s="24" t="s">
-        <v>175</v>
-      </c>
-      <c r="B56" s="24" t="s">
-        <v>209</v>
-      </c>
-      <c r="C56" s="25">
-        <v>0</v>
-      </c>
-      <c r="D56" s="26">
-        <v>0</v>
-      </c>
-      <c r="E56" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A57" s="24" t="s">
-        <v>176</v>
-      </c>
-      <c r="B57" s="24" t="s">
-        <v>210</v>
-      </c>
-      <c r="C57" s="25">
-        <v>0</v>
-      </c>
-      <c r="D57" s="26">
+      <c r="C57" s="24">
+        <v>0</v>
+      </c>
+      <c r="D57" s="25">
         <v>0</v>
       </c>
       <c r="E57" t="s">
@@ -5067,16 +5631,16 @@
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A58" s="24" t="s">
-        <v>111</v>
-      </c>
-      <c r="B58" s="24" t="s">
-        <v>113</v>
-      </c>
-      <c r="C58" s="25">
-        <v>0</v>
-      </c>
-      <c r="D58" s="26">
+      <c r="A58" s="23" t="s">
+        <v>101</v>
+      </c>
+      <c r="B58" s="23" t="s">
+        <v>102</v>
+      </c>
+      <c r="C58" s="24">
+        <v>0</v>
+      </c>
+      <c r="D58" s="25">
         <v>0</v>
       </c>
       <c r="E58" t="s">

</xml_diff>